<commit_message>
docs(qa): 第二轮 review 报告（B-10~B-15）+ 核心不变量写入 AGENTS.md
- 报告新增 B-10~B-15 六个缺陷（高 1 / 中 3 / 低 2），均含复现、根因、修复与验证方式；
  累计 15 缺陷：已修复 14、误报 1。
- 记录越权专项核查结论：15 项跨账号对抗测试全部 403/404，且**三项探针最初是误报**
  （favorites/follows/chat_read_state 返回 200/201 看着像越权，实际 handler 忽略 body 里的
  userId、以 token 身份落库）—— 判断越权要看落库归属，不能只看响应码。
- 记下一项数据决策（未擅自改）：photographers.rating/review_count 与 reviews 表脱钩
  （示例 4.9/234 vs 真实 3 条），现已改为每次新评价按事实重算，是否需要一次性回填待定。
- AGENTS.md 新增「完整性约束与核心不变量」一节：时段唯一索引、过去档期、禁止自成交、
  评价三条规则与评分重算、排序键与稳定分页、缓存键必须含 sort、本地日期不得用 toISOString、
  IDOR 现状与统一授权模式（新增接口沿用 assertSelf / ForUser / 覆盖 body userId）。
- 同时如实标注一条验证缺口：列表筛选的浏览器点击级验证未完成（agent-browser 会话 CDP 卡死），
  已由接口层 + DB 集成测试覆盖。
</commit_message>
<xml_diff>
--- a/docs/qa/2026-09-24-C端角色扮演整体测试-报告.xlsx
+++ b/docs/qa/2026-09-24-C端角色扮演整体测试-报告.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'用例结果'!$A$1:$G$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'缺陷清单'!$A$1:$K$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'缺陷清单'!$A$1:$K$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1487,7 +1487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2083,8 +2083,380 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>B-10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>同一时段可被并发重复预约（缺 DB 约束）</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>订单 / 预约核心</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>用线程屏障让 12 个 POST /bookings 同时抢同一摄影师同一 date+time</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>只应有 1 单成功，其余 409</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>7 个请求返回 201、7 条订单落在同一时段（顺序请求能正确 409，并发打不穿 —— CountConflictBookings 是先查后插的 TOCTOU）</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>bookings 表只有主键，没有任何 (photographer_id, date, time) 唯一约束；应用层检查在并发下必然失效。一位摄影师同一档期被约 7 次。</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>server/migrations/000029_integrity_constraints.up.sql + booking_service.Create</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>部分唯一索引 uniq_bookings_active_slot（WHERE status &lt;&gt; 'cancelled'，取消释放时段）+ 把 23505 映射成 409</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>已修复 — 复测 12 并发：1 个 201、11 个 409、落库 1 条</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>已修复 — 时段唯一约束（部分唯一索引）+ 23505→409</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>B-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>可以预约已经过去的日期（且预约页默认日期会落在昨天）</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>订单 / 预约核心</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>POST /bookings 传 date=2020-01-01；或本地时间早 8 点前打开预约页看默认日期</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>服务端拒绝过去档期；默认日期为本地今天</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>过去日期下单返回 201 并落库；前端用 new Date().toISOString() 取日期（UTC），东八区 00:00-08:00 会取到昨天，一进页面就默认选中过去的一天</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>服务端 Create 只校验日期格式；前端 booking/index.vue:118 用了 toISOString 取本地日期；日期选择器也没有 start 下限</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>server/internal/service/booking_service.go（isPastSlot）+ src/utils/date.ts + booking 页</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>服务端按服务器本地时区拒绝过去档期（今天是硬约束，时刻尽力而为）；前端新增本地日期工具并给 picker 加 :start</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>已修复 — 过去日期/今天已过时刻均 400</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>已修复 — 服务端拒绝过去日期/时刻；前端改用本地日期并给选择器加下限</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>B-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>摄影师可以预约自己的套餐（自成交）</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>订单 / 业务逻辑</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>以摄影师 5 的账号 POST /bookings 预约摄影师 5 自己的套餐</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>拒绝 —— 自成交无业务含义</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>201 创建成功，订单的 coser 就是该摄影师本人</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Create 只校验套餐归属与黑名单，没有比较下单人与摄影师 owner；自成交会污染单量，并为「自己给自己评价」铺路</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>server/internal/service/booking_service.go（ErrSelfBooking）</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>下单人 == 摄影师 owner 时返回 400</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>已修复 — 禁止摄影师预约自己的套餐</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>B-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>评价没有任何前置校验，且评分/评价数从不更新</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>评价 / 商家信誉</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>未与该摄影师成交过的账号 POST /reviews；或同一人对同一摄影师重复评价</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>只有已完成订单可评价，且一人一评</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>任何登录用户都能给任何摄影师评价，且可无限重复；更关键的是 photographers.rating / review_count 从不随评价更新 —— 列表显示 4.9 分 / 234 条评价，而该摄影师真实只有 3 条评价</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>ReviewService.Create 直接 INSERT；reviews 表无唯一约束；没有触发器、也没有任何聚合更新代码，两个评分字段是种子数据里的死数字</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>server/internal/service/review_service.go + repository/reviews.sql.go + 迁移 000029</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>① 校验存在已完成订单 ② 不能自评 ③ 唯一索引（photographer_id, user_id）兜重复 ④ 每次评价后按 reviews 重算评分与评价数</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>已修复 — 未成交评价 403、重复评价 409、评价成功后评分按事实重算（实测 4.3 / 3 条）</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>已修复 — 评价需已完成订单 + 一人一评 + 评分/评价数按事实重算</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>B-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>摄影师列表的筛选栏全部无效（4 个筛选返回同一结果）</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>C 端 · 摄影师列表</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>打开 摄影师 列表，依次点 热门 / 评分最高 / 接单最多 / 最新入驻</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>四种排序应给出不同顺序</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>只有高亮变化，结果完全一样</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>list.vue 的 setFilter 只改 currentFilter 就重新 loadData，而 loadData 只发 page/size；后端 List 也不接受任何排序参数（SQL 里固定 ORDER BY rating, order_count）</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>src/pages/photographer/list.vue + repository/photographers.sql.go</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>新增 sort 参数（CASE 参数绑定，非字符串拼接）并接进缓存键；同时补 p.id DESC 作为稳定 tiebreaker（排序键不唯一时 LIMIT/OFFSET 翻页会重复/漏行）</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>已修复 — 接口层与 DB 集成测试验证四种排序；演示数据恰好单调，区分度由交叉夹具数据证明</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>已修复 — 筛选键接到服务端排序（sort），并补稳定分页 tiebreaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>B-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>非会话成员也能标记别人的会话「已读」</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>聊天 / 越权（自伤）</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>以不在会话 1 的用户 POST /chat/sessions/1/read</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>403 —— 与 ListMessages / SendMessage 口径一致</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>200 {ok:true}，并给自己写了一条无意义的 chat_read_state 行</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>ChatService.MarkSessionRead 直通 repository，没有 assertParticipant（同文件另外两个入口都有）；影响仅限调用者自己的状态，无跨用户泄露</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>server/internal/service/chat_service.go</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>补 assertParticipant，handler 映射 403/404</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>已修复 — 复测 403</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>已修复 — 非会话成员标记已读改为 403</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K10"/>
+  <autoFilter ref="A1:K16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2095,7 +2467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2223,12 +2595,12 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>COUNTA(缺陷清单!A2:A10)</f>
+        <f>COUNTA(缺陷清单!A2:A16)</f>
         <v/>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>值=9</t>
+          <t>值=15</t>
         </is>
       </c>
     </row>
@@ -2239,12 +2611,12 @@
         </is>
       </c>
       <c r="B9" s="10">
-        <f>COUNTIF(缺陷清单!C2:C10,"高")</f>
+        <f>COUNTIF(缺陷清单!C2:C16,"高")</f>
         <v/>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>值=2</t>
+          <t>值=3</t>
         </is>
       </c>
     </row>
@@ -2255,12 +2627,12 @@
         </is>
       </c>
       <c r="B10" s="10">
-        <f>COUNTIF(缺陷清单!C2:C10,"中")</f>
+        <f>COUNTIF(缺陷清单!C2:C16,"中")</f>
         <v/>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>值=5</t>
+          <t>值=8</t>
         </is>
       </c>
     </row>
@@ -2271,12 +2643,12 @@
         </is>
       </c>
       <c r="B11" s="10">
-        <f>COUNTIF(缺陷清单!C2:C10,"低")</f>
+        <f>COUNTIF(缺陷清单!C2:C16,"低")</f>
         <v/>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>值=2</t>
+          <t>值=4</t>
         </is>
       </c>
     </row>
@@ -2287,12 +2659,12 @@
         </is>
       </c>
       <c r="B12" s="10">
-        <f>COUNTIF(缺陷清单!K2:K10,"已修复*")</f>
+        <f>COUNTIF(缺陷清单!K2:K16,"已修复*")</f>
         <v/>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>值=8</t>
+          <t>值=14</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2675,7 @@
         </is>
       </c>
       <c r="B13" s="10">
-        <f>COUNTIF(缺陷清单!K2:K10,"待定夺*")</f>
+        <f>COUNTIF(缺陷清单!K2:K16,"待定夺*")</f>
         <v/>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -2319,7 +2691,7 @@
         </is>
       </c>
       <c r="B14" s="10">
-        <f>COUNTIF(缺陷清单!K2:K10,"误报*")</f>
+        <f>COUNTIF(缺陷清单!K2:K16,"误报*")</f>
         <v/>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -2433,12 +2805,36 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>第二轮整体 review（2026-09-24，业务逻辑 + 核心功能）新增 B-10~B-15 六个缺陷，全部已修复并复测。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>越权面专项核查（跨账号对抗测试）：15 项「用 A 的 token 读写 B 的资源」全部 403/404 —— 订单读取与改状态、跨摄影师读接单、非本人会话读消息/发消息、收藏/关注/通知的越权写，均已正确拒绝；其中 favorites / follows / chat_read_state 三项探针最初显示 200/201，经查是**探针误报**（handler 忽略 body 里的 userId、一律用 token 身份，落库归属正确），不构成缺陷。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>待你定夺（数据决策，非缺陷）：photographers.rating / review_count 是种子数字，与 reviews 表脱钩（示例：光影行者显示 4.9 / 234 条，真实只有 3 条）。B-13 已让它们**在每次新评价时按事实重算**，所以新评价一到就会自我修正；是否要把现有数据一次性回填成真实值（评分与评价数会显著变小），属演示数据取舍，未擅自改动。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="17">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A33:C33"/>
     <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A18:C18"/>

</xml_diff>